<commit_message>
Add Illumia fixed gas offer
</commit_message>
<xml_diff>
--- a/tariffe/2026-05/residenziale/tariffe_illumia_template.xlsx
+++ b/tariffe/2026-05/residenziale/tariffe_illumia_template.xlsx
@@ -1163,7 +1163,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GAS PREMIUM FIX</t>
+          <t>A MODO TUO FIX GAS 36</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -1182,15 +1182,17 @@
           <t>€/Smc</t>
         </is>
       </c>
-      <c r="J13" s="3" t="n"/>
+      <c r="J13" s="3" t="n">
+        <v>0.55</v>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Nessuna offerta gas fissa Illumia nei PDF maggio ricevuti</t>
+          <t>Da PDF CE-ILLUMIA-A-MODO-TUO-FIX-GAS-36-RF: corrispettivo per il consumo nei primi 36 mesi 0,55 €/Smc</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1219,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GAS PREMIUM FIX</t>
+          <t>A MODO TUO FIX GAS 36</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -1236,15 +1238,17 @@
           <t>€/anno</t>
         </is>
       </c>
-      <c r="J14" s="3" t="n"/>
+      <c r="J14" s="3" t="n">
+        <v>144</v>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Nessuna offerta gas fissa Illumia nei PDF maggio ricevuti</t>
+          <t>Da PDF CE-ILLUMIA-A-MODO-TUO-FIX-GAS-36-RF: corrispettivo annuo 144 €/PDR/anno</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
     </row>

</xml_diff>